<commit_message>
Add inert TPR opening item configs
</commit_message>
<xml_diff>
--- a/jyx2/Assets/Mods/jshyl/Configs/物品.xlsx
+++ b/jyx2/Assets/Mods/jshyl/Configs/物品.xlsx
@@ -540,7 +540,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AX209"/>
+  <dimension ref="A1:AX214"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="14"/>
   <cols>
     <col width="28.36328125" customWidth="1" style="1" min="50" max="50"/>
@@ -33292,6 +33292,806 @@
       </c>
       <c r="AW209" t="inlineStr"/>
     </row>
+    <row r="210">
+      <c r="A210" t="n">
+        <v>205</v>
+      </c>
+      <c r="B210" t="inlineStr">
+        <is>
+          <t>司南针</t>
+        </is>
+      </c>
+      <c r="C210" t="inlineStr">
+        <is>
+          <t>司</t>
+        </is>
+      </c>
+      <c r="D210" t="inlineStr">
+        <is>
+          <t>QQZJ/TPR开局道具。慕容秋荻所赠行路之物，可辨方位。</t>
+        </is>
+      </c>
+      <c r="E210" t="n">
+        <v>-1</v>
+      </c>
+      <c r="F210" t="n">
+        <v>-1</v>
+      </c>
+      <c r="G210" t="n">
+        <v>-1</v>
+      </c>
+      <c r="H210" t="n">
+        <v>0</v>
+      </c>
+      <c r="I210" t="n">
+        <v>0</v>
+      </c>
+      <c r="J210" t="n">
+        <v>0</v>
+      </c>
+      <c r="K210" t="n">
+        <v>0</v>
+      </c>
+      <c r="L210" t="n">
+        <v>0</v>
+      </c>
+      <c r="M210" t="n">
+        <v>0</v>
+      </c>
+      <c r="N210" t="n">
+        <v>0</v>
+      </c>
+      <c r="O210" t="n">
+        <v>0</v>
+      </c>
+      <c r="P210" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q210" t="n">
+        <v>0</v>
+      </c>
+      <c r="R210" t="n">
+        <v>0</v>
+      </c>
+      <c r="S210" t="n">
+        <v>0</v>
+      </c>
+      <c r="T210" t="n">
+        <v>0</v>
+      </c>
+      <c r="U210" t="n">
+        <v>0</v>
+      </c>
+      <c r="V210" t="n">
+        <v>0</v>
+      </c>
+      <c r="W210" t="n">
+        <v>0</v>
+      </c>
+      <c r="X210" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y210" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z210" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA210" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB210" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC210" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD210" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE210" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF210" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG210" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH210" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI210" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ210" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK210" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL210" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM210" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN210" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO210" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP210" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ210" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR210" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS210" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT210" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU210" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AV210" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW210" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AX210" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" t="n">
+        <v>206</v>
+      </c>
+      <c r="B211" t="inlineStr">
+        <is>
+          <t>狼牙燕翎</t>
+        </is>
+      </c>
+      <c r="C211" t="inlineStr">
+        <is>
+          <t>狼</t>
+        </is>
+      </c>
+      <c r="D211" t="inlineStr">
+        <is>
+          <t>QQZJ/TPR开局道具。燕子坞家传暗记，可作江湖行走凭证。</t>
+        </is>
+      </c>
+      <c r="E211" t="n">
+        <v>-1</v>
+      </c>
+      <c r="F211" t="n">
+        <v>-1</v>
+      </c>
+      <c r="G211" t="n">
+        <v>-1</v>
+      </c>
+      <c r="H211" t="n">
+        <v>0</v>
+      </c>
+      <c r="I211" t="n">
+        <v>0</v>
+      </c>
+      <c r="J211" t="n">
+        <v>0</v>
+      </c>
+      <c r="K211" t="n">
+        <v>0</v>
+      </c>
+      <c r="L211" t="n">
+        <v>0</v>
+      </c>
+      <c r="M211" t="n">
+        <v>0</v>
+      </c>
+      <c r="N211" t="n">
+        <v>0</v>
+      </c>
+      <c r="O211" t="n">
+        <v>0</v>
+      </c>
+      <c r="P211" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q211" t="n">
+        <v>0</v>
+      </c>
+      <c r="R211" t="n">
+        <v>0</v>
+      </c>
+      <c r="S211" t="n">
+        <v>0</v>
+      </c>
+      <c r="T211" t="n">
+        <v>0</v>
+      </c>
+      <c r="U211" t="n">
+        <v>0</v>
+      </c>
+      <c r="V211" t="n">
+        <v>0</v>
+      </c>
+      <c r="W211" t="n">
+        <v>0</v>
+      </c>
+      <c r="X211" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y211" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z211" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA211" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB211" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC211" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD211" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE211" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF211" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG211" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH211" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI211" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ211" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK211" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL211" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM211" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN211" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO211" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP211" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ211" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR211" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS211" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT211" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU211" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AV211" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW211" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AX211" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" t="n">
+        <v>207</v>
+      </c>
+      <c r="B212" t="inlineStr">
+        <is>
+          <t>秦皇照骨镜</t>
+        </is>
+      </c>
+      <c r="C212" t="inlineStr">
+        <is>
+          <t>秦</t>
+        </is>
+      </c>
+      <c r="D212" t="inlineStr">
+        <is>
+          <t>QQZJ/TPR开局道具。古镜一面，据说可照见机关与遗迹线索。</t>
+        </is>
+      </c>
+      <c r="E212" t="n">
+        <v>-1</v>
+      </c>
+      <c r="F212" t="n">
+        <v>-1</v>
+      </c>
+      <c r="G212" t="n">
+        <v>-1</v>
+      </c>
+      <c r="H212" t="n">
+        <v>0</v>
+      </c>
+      <c r="I212" t="n">
+        <v>0</v>
+      </c>
+      <c r="J212" t="n">
+        <v>0</v>
+      </c>
+      <c r="K212" t="n">
+        <v>0</v>
+      </c>
+      <c r="L212" t="n">
+        <v>0</v>
+      </c>
+      <c r="M212" t="n">
+        <v>0</v>
+      </c>
+      <c r="N212" t="n">
+        <v>0</v>
+      </c>
+      <c r="O212" t="n">
+        <v>0</v>
+      </c>
+      <c r="P212" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q212" t="n">
+        <v>0</v>
+      </c>
+      <c r="R212" t="n">
+        <v>0</v>
+      </c>
+      <c r="S212" t="n">
+        <v>0</v>
+      </c>
+      <c r="T212" t="n">
+        <v>0</v>
+      </c>
+      <c r="U212" t="n">
+        <v>0</v>
+      </c>
+      <c r="V212" t="n">
+        <v>0</v>
+      </c>
+      <c r="W212" t="n">
+        <v>0</v>
+      </c>
+      <c r="X212" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y212" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z212" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA212" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB212" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC212" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD212" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE212" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF212" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG212" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH212" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI212" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ212" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK212" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL212" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM212" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN212" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO212" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP212" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ212" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR212" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS212" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT212" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU212" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AV212" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW212" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AX212" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="213">
+      <c r="A213" t="n">
+        <v>208</v>
+      </c>
+      <c r="B213" t="inlineStr">
+        <is>
+          <t>洛阳铲</t>
+        </is>
+      </c>
+      <c r="C213" t="inlineStr">
+        <is>
+          <t>铲</t>
+        </is>
+      </c>
+      <c r="D213" t="inlineStr">
+        <is>
+          <t>QQZJ/TPR开局道具。探墓寻物所用器具。</t>
+        </is>
+      </c>
+      <c r="E213" t="n">
+        <v>-1</v>
+      </c>
+      <c r="F213" t="n">
+        <v>-1</v>
+      </c>
+      <c r="G213" t="n">
+        <v>-1</v>
+      </c>
+      <c r="H213" t="n">
+        <v>0</v>
+      </c>
+      <c r="I213" t="n">
+        <v>0</v>
+      </c>
+      <c r="J213" t="n">
+        <v>0</v>
+      </c>
+      <c r="K213" t="n">
+        <v>0</v>
+      </c>
+      <c r="L213" t="n">
+        <v>0</v>
+      </c>
+      <c r="M213" t="n">
+        <v>0</v>
+      </c>
+      <c r="N213" t="n">
+        <v>0</v>
+      </c>
+      <c r="O213" t="n">
+        <v>0</v>
+      </c>
+      <c r="P213" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q213" t="n">
+        <v>0</v>
+      </c>
+      <c r="R213" t="n">
+        <v>0</v>
+      </c>
+      <c r="S213" t="n">
+        <v>0</v>
+      </c>
+      <c r="T213" t="n">
+        <v>0</v>
+      </c>
+      <c r="U213" t="n">
+        <v>0</v>
+      </c>
+      <c r="V213" t="n">
+        <v>0</v>
+      </c>
+      <c r="W213" t="n">
+        <v>0</v>
+      </c>
+      <c r="X213" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y213" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z213" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA213" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB213" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC213" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD213" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE213" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF213" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG213" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH213" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI213" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ213" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK213" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL213" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM213" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN213" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO213" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP213" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ213" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR213" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS213" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT213" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU213" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AV213" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW213" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AX213" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" t="n">
+        <v>209</v>
+      </c>
+      <c r="B214" t="inlineStr">
+        <is>
+          <t>海月清辉</t>
+        </is>
+      </c>
+      <c r="C214" t="inlineStr">
+        <is>
+          <t>海</t>
+        </is>
+      </c>
+      <c r="D214" t="inlineStr">
+        <is>
+          <t>QQZJ/TPR开局道具。还施水阁所藏清雅珍物。</t>
+        </is>
+      </c>
+      <c r="E214" t="n">
+        <v>-1</v>
+      </c>
+      <c r="F214" t="n">
+        <v>-1</v>
+      </c>
+      <c r="G214" t="n">
+        <v>-1</v>
+      </c>
+      <c r="H214" t="n">
+        <v>0</v>
+      </c>
+      <c r="I214" t="n">
+        <v>0</v>
+      </c>
+      <c r="J214" t="n">
+        <v>0</v>
+      </c>
+      <c r="K214" t="n">
+        <v>0</v>
+      </c>
+      <c r="L214" t="n">
+        <v>0</v>
+      </c>
+      <c r="M214" t="n">
+        <v>0</v>
+      </c>
+      <c r="N214" t="n">
+        <v>0</v>
+      </c>
+      <c r="O214" t="n">
+        <v>0</v>
+      </c>
+      <c r="P214" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q214" t="n">
+        <v>0</v>
+      </c>
+      <c r="R214" t="n">
+        <v>0</v>
+      </c>
+      <c r="S214" t="n">
+        <v>0</v>
+      </c>
+      <c r="T214" t="n">
+        <v>0</v>
+      </c>
+      <c r="U214" t="n">
+        <v>0</v>
+      </c>
+      <c r="V214" t="n">
+        <v>0</v>
+      </c>
+      <c r="W214" t="n">
+        <v>0</v>
+      </c>
+      <c r="X214" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y214" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z214" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA214" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB214" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC214" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD214" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE214" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF214" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG214" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH214" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI214" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ214" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK214" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL214" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM214" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN214" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO214" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP214" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ214" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR214" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS214" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT214" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU214" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AV214" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW214" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AX214" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" paperSize="9" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>

<commit_message>
Add opening medicine item configs
</commit_message>
<xml_diff>
--- a/jyx2/Assets/Mods/jshyl/Configs/物品.xlsx
+++ b/jyx2/Assets/Mods/jshyl/Configs/物品.xlsx
@@ -111,7 +111,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -127,6 +127,7 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="5">
     <cellStyle name="常规" xfId="0" builtinId="0"/>
@@ -540,7 +541,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AX214"/>
+  <dimension ref="A1:AX218"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="14"/>
   <cols>
     <col width="28.36328125" customWidth="1" style="1" min="50" max="50"/>
@@ -32525,1572 +32526,2176 @@
       <c r="AX204" s="5" t="n"/>
     </row>
     <row r="205">
-      <c r="A205" t="n">
+      <c r="A205" s="0" t="n">
         <v>200</v>
       </c>
-      <c r="B205" t="inlineStr">
+      <c r="B205" s="0" t="inlineStr">
         <is>
           <t>越女剑谱</t>
         </is>
       </c>
-      <c r="C205" t="inlineStr">
+      <c r="C205" s="0" t="inlineStr">
         <is>
           <t>越</t>
         </is>
       </c>
-      <c r="D205" t="inlineStr">
+      <c r="D205" s="0" t="inlineStr">
         <is>
           <t>越女剑线奖励秘籍，修习越女剑法。</t>
         </is>
       </c>
-      <c r="E205" t="n">
+      <c r="E205" s="0" t="n">
         <v>61</v>
       </c>
-      <c r="F205" t="n">
-        <v>-1</v>
-      </c>
-      <c r="G205" t="n">
-        <v>-1</v>
-      </c>
-      <c r="H205" t="n">
+      <c r="F205" s="0" t="n">
+        <v>-1</v>
+      </c>
+      <c r="G205" s="0" t="n">
+        <v>-1</v>
+      </c>
+      <c r="H205" s="0" t="n">
         <v>2</v>
       </c>
-      <c r="I205" t="n">
-        <v>0</v>
-      </c>
-      <c r="J205" t="n">
-        <v>0</v>
-      </c>
-      <c r="K205" t="n">
-        <v>0</v>
-      </c>
-      <c r="L205" t="n">
-        <v>0</v>
-      </c>
-      <c r="M205" t="n">
-        <v>-1</v>
-      </c>
-      <c r="N205" t="n">
-        <v>0</v>
-      </c>
-      <c r="O205" t="n">
-        <v>0</v>
-      </c>
-      <c r="P205" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q205" t="n">
-        <v>0</v>
-      </c>
-      <c r="R205" t="n">
-        <v>0</v>
-      </c>
-      <c r="S205" t="n">
-        <v>0</v>
-      </c>
-      <c r="T205" t="n">
-        <v>0</v>
-      </c>
-      <c r="U205" t="n">
-        <v>0</v>
-      </c>
-      <c r="V205" t="n">
+      <c r="I205" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="J205" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="K205" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="L205" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="M205" s="0" t="n">
+        <v>-1</v>
+      </c>
+      <c r="N205" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="O205" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="P205" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q205" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="R205" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="S205" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="T205" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="U205" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="V205" s="0" t="n">
         <v>10</v>
       </c>
-      <c r="W205" t="n">
-        <v>0</v>
-      </c>
-      <c r="X205" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y205" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z205" t="n">
-        <v>0</v>
-      </c>
-      <c r="AA205" t="n">
-        <v>0</v>
-      </c>
-      <c r="AB205" t="n">
-        <v>0</v>
-      </c>
-      <c r="AC205" t="n">
-        <v>0</v>
-      </c>
-      <c r="AD205" t="n">
-        <v>-1</v>
-      </c>
-      <c r="AE205" t="n">
+      <c r="W205" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="X205" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y205" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z205" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA205" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB205" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC205" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD205" s="0" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AE205" s="0" t="n">
         <v>2</v>
       </c>
-      <c r="AF205" t="n">
-        <v>0</v>
-      </c>
-      <c r="AG205" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH205" t="n">
-        <v>0</v>
-      </c>
-      <c r="AI205" t="n">
-        <v>0</v>
-      </c>
-      <c r="AJ205" t="n">
-        <v>0</v>
-      </c>
-      <c r="AK205" t="n">
-        <v>0</v>
-      </c>
-      <c r="AL205" t="n">
-        <v>0</v>
-      </c>
-      <c r="AM205" t="n">
+      <c r="AF205" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG205" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH205" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI205" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ205" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK205" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL205" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM205" s="0" t="n">
         <v>60</v>
       </c>
-      <c r="AN205" t="n">
-        <v>0</v>
-      </c>
-      <c r="AO205" t="n">
-        <v>0</v>
-      </c>
-      <c r="AP205" t="n">
-        <v>0</v>
-      </c>
-      <c r="AQ205" t="n">
-        <v>0</v>
-      </c>
-      <c r="AR205" t="n">
+      <c r="AN205" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO205" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP205" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ205" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR205" s="0" t="n">
         <v>60</v>
       </c>
-      <c r="AS205" t="n">
+      <c r="AS205" s="0" t="n">
         <v>200</v>
       </c>
-      <c r="AT205" t="n">
-        <v>-1</v>
-      </c>
-      <c r="AU205" t="n">
-        <v>0</v>
-      </c>
-      <c r="AV205" t="n">
-        <v>-1</v>
-      </c>
-      <c r="AW205" t="inlineStr"/>
+      <c r="AT205" s="0" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AU205" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV205" s="0" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AW205" s="0" t="inlineStr"/>
     </row>
     <row r="206">
-      <c r="A206" t="n">
+      <c r="A206" s="0" t="n">
         <v>201</v>
       </c>
-      <c r="B206" t="inlineStr">
+      <c r="B206" s="0" t="inlineStr">
         <is>
           <t>瑶池仙袖</t>
         </is>
       </c>
-      <c r="C206" t="inlineStr">
+      <c r="C206" s="0" t="inlineStr">
         <is>
           <t>瑶</t>
         </is>
       </c>
-      <c r="D206" t="inlineStr">
+      <c r="D206" s="0" t="inlineStr">
         <is>
           <t>九天玄女所遗仙衣，轻灵而护体。</t>
         </is>
       </c>
-      <c r="E206" t="n">
-        <v>-1</v>
-      </c>
-      <c r="F206" t="n">
-        <v>-1</v>
-      </c>
-      <c r="G206" t="n">
+      <c r="E206" s="0" t="n">
+        <v>-1</v>
+      </c>
+      <c r="F206" s="0" t="n">
+        <v>-1</v>
+      </c>
+      <c r="G206" s="0" t="n">
         <v>1</v>
       </c>
-      <c r="H206" t="n">
+      <c r="H206" s="0" t="n">
         <v>1</v>
       </c>
-      <c r="I206" t="n">
-        <v>0</v>
-      </c>
-      <c r="J206" t="n">
+      <c r="I206" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="J206" s="0" t="n">
         <v>100</v>
       </c>
-      <c r="K206" t="n">
-        <v>0</v>
-      </c>
-      <c r="L206" t="n">
-        <v>0</v>
-      </c>
-      <c r="M206" t="n">
-        <v>0</v>
-      </c>
-      <c r="N206" t="n">
-        <v>0</v>
-      </c>
-      <c r="O206" t="n">
+      <c r="K206" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="L206" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="M206" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="N206" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="O206" s="0" t="n">
         <v>80</v>
       </c>
-      <c r="P206" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q206" t="n">
+      <c r="P206" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q206" s="0" t="n">
         <v>20</v>
       </c>
-      <c r="R206" t="n">
+      <c r="R206" s="0" t="n">
         <v>30</v>
       </c>
-      <c r="S206" t="n">
-        <v>0</v>
-      </c>
-      <c r="T206" t="n">
-        <v>0</v>
-      </c>
-      <c r="U206" t="n">
-        <v>0</v>
-      </c>
-      <c r="V206" t="n">
+      <c r="S206" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="T206" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="U206" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="V206" s="0" t="n">
         <v>20</v>
       </c>
-      <c r="W206" t="n">
-        <v>0</v>
-      </c>
-      <c r="X206" t="n">
+      <c r="W206" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="X206" s="0" t="n">
         <v>10</v>
       </c>
-      <c r="Y206" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z206" t="n">
-        <v>0</v>
-      </c>
-      <c r="AA206" t="n">
-        <v>0</v>
-      </c>
-      <c r="AB206" t="n">
+      <c r="Y206" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z206" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA206" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB206" s="0" t="n">
         <v>5</v>
       </c>
-      <c r="AC206" t="n">
-        <v>0</v>
-      </c>
-      <c r="AD206" t="n">
-        <v>-1</v>
-      </c>
-      <c r="AE206" t="n">
+      <c r="AC206" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD206" s="0" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AE206" s="0" t="n">
         <v>2</v>
       </c>
-      <c r="AF206" t="n">
-        <v>0</v>
-      </c>
-      <c r="AG206" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH206" t="n">
-        <v>0</v>
-      </c>
-      <c r="AI206" t="n">
-        <v>0</v>
-      </c>
-      <c r="AJ206" t="n">
-        <v>0</v>
-      </c>
-      <c r="AK206" t="n">
-        <v>0</v>
-      </c>
-      <c r="AL206" t="n">
-        <v>0</v>
-      </c>
-      <c r="AM206" t="n">
-        <v>0</v>
-      </c>
-      <c r="AN206" t="n">
-        <v>0</v>
-      </c>
-      <c r="AO206" t="n">
-        <v>0</v>
-      </c>
-      <c r="AP206" t="n">
-        <v>0</v>
-      </c>
-      <c r="AQ206" t="n">
-        <v>0</v>
-      </c>
-      <c r="AR206" t="n">
+      <c r="AF206" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG206" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH206" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI206" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ206" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK206" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL206" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM206" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN206" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO206" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP206" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ206" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR206" s="0" t="n">
         <v>80</v>
       </c>
-      <c r="AS206" t="n">
-        <v>0</v>
-      </c>
-      <c r="AT206" t="n">
-        <v>-1</v>
-      </c>
-      <c r="AU206" t="n">
-        <v>0</v>
-      </c>
-      <c r="AV206" t="n">
-        <v>-1</v>
-      </c>
-      <c r="AW206" t="inlineStr"/>
+      <c r="AS206" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT206" s="0" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AU206" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV206" s="0" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AW206" s="0" t="inlineStr"/>
     </row>
     <row r="207">
-      <c r="A207" t="n">
+      <c r="A207" s="0" t="n">
         <v>202</v>
       </c>
-      <c r="B207" t="inlineStr">
+      <c r="B207" s="0" t="inlineStr">
         <is>
           <t>长生诀</t>
         </is>
       </c>
-      <c r="C207" t="inlineStr">
+      <c r="C207" s="0" t="inlineStr">
         <is>
           <t>长</t>
         </is>
       </c>
-      <c r="D207" t="inlineStr">
+      <c r="D207" s="0" t="inlineStr">
         <is>
           <t>玄门养生奇书，提升生命与内力根基。</t>
         </is>
       </c>
-      <c r="E207" t="n">
-        <v>-1</v>
-      </c>
-      <c r="F207" t="n">
-        <v>-1</v>
-      </c>
-      <c r="G207" t="n">
-        <v>-1</v>
-      </c>
-      <c r="H207" t="n">
+      <c r="E207" s="0" t="n">
+        <v>-1</v>
+      </c>
+      <c r="F207" s="0" t="n">
+        <v>-1</v>
+      </c>
+      <c r="G207" s="0" t="n">
+        <v>-1</v>
+      </c>
+      <c r="H207" s="0" t="n">
         <v>2</v>
       </c>
-      <c r="I207" t="n">
-        <v>0</v>
-      </c>
-      <c r="J207" t="n">
+      <c r="I207" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="J207" s="0" t="n">
         <v>100</v>
       </c>
-      <c r="K207" t="n">
-        <v>0</v>
-      </c>
-      <c r="L207" t="n">
-        <v>0</v>
-      </c>
-      <c r="M207" t="n">
-        <v>-1</v>
-      </c>
-      <c r="N207" t="n">
-        <v>0</v>
-      </c>
-      <c r="O207" t="n">
+      <c r="K207" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="L207" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="M207" s="0" t="n">
+        <v>-1</v>
+      </c>
+      <c r="N207" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="O207" s="0" t="n">
         <v>100</v>
       </c>
-      <c r="P207" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q207" t="n">
-        <v>0</v>
-      </c>
-      <c r="R207" t="n">
+      <c r="P207" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q207" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="R207" s="0" t="n">
         <v>10</v>
       </c>
-      <c r="S207" t="n">
-        <v>0</v>
-      </c>
-      <c r="T207" t="n">
-        <v>0</v>
-      </c>
-      <c r="U207" t="n">
-        <v>0</v>
-      </c>
-      <c r="V207" t="n">
+      <c r="S207" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="T207" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="U207" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="V207" s="0" t="n">
         <v>10</v>
       </c>
-      <c r="W207" t="n">
-        <v>0</v>
-      </c>
-      <c r="X207" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y207" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z207" t="n">
-        <v>0</v>
-      </c>
-      <c r="AA207" t="n">
-        <v>0</v>
-      </c>
-      <c r="AB207" t="n">
+      <c r="W207" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="X207" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y207" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z207" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA207" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB207" s="0" t="n">
         <v>10</v>
       </c>
-      <c r="AC207" t="n">
-        <v>0</v>
-      </c>
-      <c r="AD207" t="n">
-        <v>-1</v>
-      </c>
-      <c r="AE207" t="n">
+      <c r="AC207" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD207" s="0" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AE207" s="0" t="n">
         <v>2</v>
       </c>
-      <c r="AF207" t="n">
-        <v>0</v>
-      </c>
-      <c r="AG207" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH207" t="n">
-        <v>0</v>
-      </c>
-      <c r="AI207" t="n">
-        <v>0</v>
-      </c>
-      <c r="AJ207" t="n">
-        <v>0</v>
-      </c>
-      <c r="AK207" t="n">
-        <v>0</v>
-      </c>
-      <c r="AL207" t="n">
-        <v>0</v>
-      </c>
-      <c r="AM207" t="n">
-        <v>0</v>
-      </c>
-      <c r="AN207" t="n">
-        <v>0</v>
-      </c>
-      <c r="AO207" t="n">
-        <v>0</v>
-      </c>
-      <c r="AP207" t="n">
-        <v>0</v>
-      </c>
-      <c r="AQ207" t="n">
-        <v>0</v>
-      </c>
-      <c r="AR207" t="n">
+      <c r="AF207" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG207" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH207" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI207" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ207" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK207" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL207" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM207" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN207" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO207" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP207" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ207" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR207" s="0" t="n">
         <v>70</v>
       </c>
-      <c r="AS207" t="n">
+      <c r="AS207" s="0" t="n">
         <v>300</v>
       </c>
-      <c r="AT207" t="n">
-        <v>-1</v>
-      </c>
-      <c r="AU207" t="n">
-        <v>0</v>
-      </c>
-      <c r="AV207" t="n">
-        <v>-1</v>
-      </c>
-      <c r="AW207" t="inlineStr"/>
+      <c r="AT207" s="0" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AU207" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV207" s="0" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AW207" s="0" t="inlineStr"/>
     </row>
     <row r="208">
-      <c r="A208" t="n">
+      <c r="A208" s="0" t="n">
         <v>203</v>
       </c>
-      <c r="B208" t="inlineStr">
+      <c r="B208" s="0" t="inlineStr">
         <is>
           <t>天元剑气诀</t>
         </is>
       </c>
-      <c r="C208" t="inlineStr">
+      <c r="C208" s="0" t="inlineStr">
         <is>
           <t>天</t>
         </is>
       </c>
-      <c r="D208" t="inlineStr">
+      <c r="D208" s="0" t="inlineStr">
         <is>
           <t>玄女剑意化成的特技秘本，偏重御剑与武常。</t>
         </is>
       </c>
-      <c r="E208" t="n">
-        <v>-1</v>
-      </c>
-      <c r="F208" t="n">
-        <v>-1</v>
-      </c>
-      <c r="G208" t="n">
-        <v>-1</v>
-      </c>
-      <c r="H208" t="n">
+      <c r="E208" s="0" t="n">
+        <v>-1</v>
+      </c>
+      <c r="F208" s="0" t="n">
+        <v>-1</v>
+      </c>
+      <c r="G208" s="0" t="n">
+        <v>-1</v>
+      </c>
+      <c r="H208" s="0" t="n">
         <v>2</v>
       </c>
-      <c r="I208" t="n">
-        <v>0</v>
-      </c>
-      <c r="J208" t="n">
-        <v>0</v>
-      </c>
-      <c r="K208" t="n">
-        <v>0</v>
-      </c>
-      <c r="L208" t="n">
-        <v>0</v>
-      </c>
-      <c r="M208" t="n">
-        <v>-1</v>
-      </c>
-      <c r="N208" t="n">
-        <v>0</v>
-      </c>
-      <c r="O208" t="n">
-        <v>0</v>
-      </c>
-      <c r="P208" t="n">
+      <c r="I208" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="J208" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="K208" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="L208" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="M208" s="0" t="n">
+        <v>-1</v>
+      </c>
+      <c r="N208" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="O208" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="P208" s="0" t="n">
         <v>10</v>
       </c>
-      <c r="Q208" t="n">
-        <v>0</v>
-      </c>
-      <c r="R208" t="n">
-        <v>0</v>
-      </c>
-      <c r="S208" t="n">
-        <v>0</v>
-      </c>
-      <c r="T208" t="n">
-        <v>0</v>
-      </c>
-      <c r="U208" t="n">
-        <v>0</v>
-      </c>
-      <c r="V208" t="n">
-        <v>0</v>
-      </c>
-      <c r="W208" t="n">
-        <v>0</v>
-      </c>
-      <c r="X208" t="n">
+      <c r="Q208" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="R208" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="S208" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="T208" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="U208" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="V208" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="W208" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="X208" s="0" t="n">
         <v>20</v>
       </c>
-      <c r="Y208" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z208" t="n">
-        <v>0</v>
-      </c>
-      <c r="AA208" t="n">
-        <v>0</v>
-      </c>
-      <c r="AB208" t="n">
-        <v>0</v>
-      </c>
-      <c r="AC208" t="n">
+      <c r="Y208" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z208" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA208" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB208" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC208" s="0" t="n">
         <v>20</v>
       </c>
-      <c r="AD208" t="n">
-        <v>0</v>
-      </c>
-      <c r="AE208" t="n">
-        <v>-1</v>
-      </c>
-      <c r="AF208" t="n">
+      <c r="AD208" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE208" s="0" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AF208" s="0" t="n">
         <v>2</v>
       </c>
-      <c r="AG208" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH208" t="n">
-        <v>0</v>
-      </c>
-      <c r="AI208" t="n">
-        <v>0</v>
-      </c>
-      <c r="AJ208" t="n">
-        <v>0</v>
-      </c>
-      <c r="AK208" t="n">
-        <v>0</v>
-      </c>
-      <c r="AL208" t="n">
-        <v>0</v>
-      </c>
-      <c r="AM208" t="n">
-        <v>0</v>
-      </c>
-      <c r="AN208" t="n">
+      <c r="AG208" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH208" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI208" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ208" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK208" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL208" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM208" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN208" s="0" t="n">
         <v>70</v>
       </c>
-      <c r="AO208" t="n">
-        <v>0</v>
-      </c>
-      <c r="AP208" t="n">
-        <v>0</v>
-      </c>
-      <c r="AQ208" t="n">
-        <v>0</v>
-      </c>
-      <c r="AR208" t="n">
-        <v>0</v>
-      </c>
-      <c r="AS208" t="n">
+      <c r="AO208" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP208" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ208" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR208" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS208" s="0" t="n">
         <v>85</v>
       </c>
-      <c r="AT208" t="n">
+      <c r="AT208" s="0" t="n">
         <v>500</v>
       </c>
-      <c r="AU208" t="n">
-        <v>-1</v>
-      </c>
-      <c r="AV208" t="n">
-        <v>0</v>
-      </c>
-      <c r="AW208" t="n">
-        <v>-1</v>
-      </c>
-      <c r="AX208" t="inlineStr"/>
+      <c r="AU208" s="0" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AV208" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW208" s="0" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AX208" s="0" t="inlineStr"/>
     </row>
     <row r="209">
-      <c r="A209" t="n">
+      <c r="A209" s="0" t="n">
         <v>204</v>
       </c>
-      <c r="B209" t="inlineStr">
+      <c r="B209" s="0" t="inlineStr">
         <is>
           <t>玄女剑</t>
         </is>
       </c>
-      <c r="C209" t="inlineStr">
+      <c r="C209" s="0" t="inlineStr">
         <is>
           <t>玄</t>
         </is>
       </c>
-      <c r="D209" t="inlineStr">
+      <c r="D209" s="0" t="inlineStr">
         <is>
           <t>仿九天玄女遗剑设置的样例神兵。</t>
         </is>
       </c>
-      <c r="E209" t="n">
-        <v>-1</v>
-      </c>
-      <c r="F209" t="n">
-        <v>-1</v>
-      </c>
-      <c r="G209" t="n">
-        <v>0</v>
-      </c>
-      <c r="H209" t="n">
+      <c r="E209" s="0" t="n">
+        <v>-1</v>
+      </c>
+      <c r="F209" s="0" t="n">
+        <v>-1</v>
+      </c>
+      <c r="G209" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="H209" s="0" t="n">
         <v>1</v>
       </c>
-      <c r="I209" t="n">
-        <v>0</v>
-      </c>
-      <c r="J209" t="n">
-        <v>0</v>
-      </c>
-      <c r="K209" t="n">
-        <v>0</v>
-      </c>
-      <c r="L209" t="n">
-        <v>0</v>
-      </c>
-      <c r="M209" t="n">
-        <v>0</v>
-      </c>
-      <c r="N209" t="n">
-        <v>0</v>
-      </c>
-      <c r="O209" t="n">
-        <v>0</v>
-      </c>
-      <c r="P209" t="n">
+      <c r="I209" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="J209" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="K209" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="L209" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="M209" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="N209" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="O209" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="P209" s="0" t="n">
         <v>25</v>
       </c>
-      <c r="Q209" t="n">
+      <c r="Q209" s="0" t="n">
         <v>10</v>
       </c>
-      <c r="R209" t="n">
-        <v>0</v>
-      </c>
-      <c r="S209" t="n">
-        <v>0</v>
-      </c>
-      <c r="T209" t="n">
-        <v>0</v>
-      </c>
-      <c r="U209" t="n">
-        <v>0</v>
-      </c>
-      <c r="V209" t="n">
-        <v>0</v>
-      </c>
-      <c r="W209" t="n">
+      <c r="R209" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="S209" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="T209" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="U209" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="V209" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="W209" s="0" t="n">
         <v>20</v>
       </c>
-      <c r="X209" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y209" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z209" t="n">
-        <v>0</v>
-      </c>
-      <c r="AA209" t="n">
-        <v>0</v>
-      </c>
-      <c r="AB209" t="n">
-        <v>0</v>
-      </c>
-      <c r="AC209" t="n">
-        <v>0</v>
-      </c>
-      <c r="AD209" t="n">
-        <v>-1</v>
-      </c>
-      <c r="AE209" t="n">
+      <c r="X209" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y209" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z209" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA209" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB209" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC209" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD209" s="0" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AE209" s="0" t="n">
         <v>2</v>
       </c>
-      <c r="AF209" t="n">
-        <v>0</v>
-      </c>
-      <c r="AG209" t="n">
+      <c r="AF209" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG209" s="0" t="n">
         <v>80</v>
       </c>
-      <c r="AH209" t="n">
-        <v>0</v>
-      </c>
-      <c r="AI209" t="n">
-        <v>0</v>
-      </c>
-      <c r="AJ209" t="n">
-        <v>0</v>
-      </c>
-      <c r="AK209" t="n">
-        <v>0</v>
-      </c>
-      <c r="AL209" t="n">
-        <v>0</v>
-      </c>
-      <c r="AM209" t="n">
+      <c r="AH209" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI209" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ209" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK209" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL209" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM209" s="0" t="n">
         <v>80</v>
       </c>
-      <c r="AN209" t="n">
-        <v>0</v>
-      </c>
-      <c r="AO209" t="n">
-        <v>0</v>
-      </c>
-      <c r="AP209" t="n">
-        <v>0</v>
-      </c>
-      <c r="AQ209" t="n">
-        <v>0</v>
-      </c>
-      <c r="AR209" t="n">
-        <v>0</v>
-      </c>
-      <c r="AS209" t="n">
-        <v>0</v>
-      </c>
-      <c r="AT209" t="n">
-        <v>-1</v>
-      </c>
-      <c r="AU209" t="n">
-        <v>0</v>
-      </c>
-      <c r="AV209" t="n">
-        <v>-1</v>
-      </c>
-      <c r="AW209" t="inlineStr"/>
+      <c r="AN209" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO209" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP209" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ209" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR209" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS209" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT209" s="0" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AU209" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV209" s="0" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AW209" s="0" t="inlineStr"/>
     </row>
     <row r="210">
-      <c r="A210" t="n">
+      <c r="A210" s="0" t="n">
         <v>205</v>
       </c>
-      <c r="B210" t="inlineStr">
+      <c r="B210" s="0" t="inlineStr">
         <is>
           <t>司南针</t>
         </is>
       </c>
-      <c r="C210" t="inlineStr">
+      <c r="C210" s="0" t="inlineStr">
         <is>
           <t>司</t>
         </is>
       </c>
-      <c r="D210" t="inlineStr">
+      <c r="D210" s="0" t="inlineStr">
         <is>
           <t>QQZJ/TPR开局道具。慕容秋荻所赠行路之物，可辨方位。</t>
         </is>
       </c>
-      <c r="E210" t="n">
-        <v>-1</v>
-      </c>
-      <c r="F210" t="n">
-        <v>-1</v>
-      </c>
-      <c r="G210" t="n">
-        <v>-1</v>
-      </c>
-      <c r="H210" t="n">
-        <v>0</v>
-      </c>
-      <c r="I210" t="n">
-        <v>0</v>
-      </c>
-      <c r="J210" t="n">
-        <v>0</v>
-      </c>
-      <c r="K210" t="n">
-        <v>0</v>
-      </c>
-      <c r="L210" t="n">
-        <v>0</v>
-      </c>
-      <c r="M210" t="n">
-        <v>0</v>
-      </c>
-      <c r="N210" t="n">
-        <v>0</v>
-      </c>
-      <c r="O210" t="n">
-        <v>0</v>
-      </c>
-      <c r="P210" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q210" t="n">
-        <v>0</v>
-      </c>
-      <c r="R210" t="n">
-        <v>0</v>
-      </c>
-      <c r="S210" t="n">
-        <v>0</v>
-      </c>
-      <c r="T210" t="n">
-        <v>0</v>
-      </c>
-      <c r="U210" t="n">
-        <v>0</v>
-      </c>
-      <c r="V210" t="n">
-        <v>0</v>
-      </c>
-      <c r="W210" t="n">
-        <v>0</v>
-      </c>
-      <c r="X210" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y210" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z210" t="n">
-        <v>0</v>
-      </c>
-      <c r="AA210" t="n">
-        <v>0</v>
-      </c>
-      <c r="AB210" t="n">
-        <v>0</v>
-      </c>
-      <c r="AC210" t="n">
-        <v>0</v>
-      </c>
-      <c r="AD210" t="n">
-        <v>0</v>
-      </c>
-      <c r="AE210" t="n">
-        <v>0</v>
-      </c>
-      <c r="AF210" t="n">
-        <v>0</v>
-      </c>
-      <c r="AG210" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH210" t="n">
-        <v>0</v>
-      </c>
-      <c r="AI210" t="n">
-        <v>0</v>
-      </c>
-      <c r="AJ210" t="n">
-        <v>0</v>
-      </c>
-      <c r="AK210" t="n">
-        <v>0</v>
-      </c>
-      <c r="AL210" t="n">
-        <v>0</v>
-      </c>
-      <c r="AM210" t="n">
-        <v>0</v>
-      </c>
-      <c r="AN210" t="n">
-        <v>0</v>
-      </c>
-      <c r="AO210" t="n">
-        <v>0</v>
-      </c>
-      <c r="AP210" t="n">
-        <v>0</v>
-      </c>
-      <c r="AQ210" t="n">
-        <v>0</v>
-      </c>
-      <c r="AR210" t="n">
-        <v>0</v>
-      </c>
-      <c r="AS210" t="n">
-        <v>0</v>
-      </c>
-      <c r="AT210" t="n">
-        <v>0</v>
-      </c>
-      <c r="AU210" t="n">
-        <v>-1</v>
-      </c>
-      <c r="AV210" t="n">
-        <v>0</v>
-      </c>
-      <c r="AW210" t="n">
-        <v>-1</v>
-      </c>
-      <c r="AX210" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
+      <c r="E210" s="0" t="n">
+        <v>-1</v>
+      </c>
+      <c r="F210" s="0" t="n">
+        <v>-1</v>
+      </c>
+      <c r="G210" s="0" t="n">
+        <v>-1</v>
+      </c>
+      <c r="H210" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="I210" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="J210" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="K210" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="L210" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="M210" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="N210" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="O210" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="P210" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q210" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="R210" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="S210" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="T210" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="U210" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="V210" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="W210" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="X210" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y210" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z210" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA210" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB210" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC210" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD210" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE210" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF210" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG210" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH210" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI210" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ210" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK210" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL210" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM210" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN210" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO210" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP210" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ210" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR210" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS210" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT210" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU210" s="0" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AV210" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW210" s="0" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AX210" s="0" t="inlineStr"/>
     </row>
     <row r="211">
-      <c r="A211" t="n">
+      <c r="A211" s="0" t="n">
         <v>206</v>
       </c>
-      <c r="B211" t="inlineStr">
+      <c r="B211" s="0" t="inlineStr">
         <is>
           <t>狼牙燕翎</t>
         </is>
       </c>
-      <c r="C211" t="inlineStr">
+      <c r="C211" s="0" t="inlineStr">
         <is>
           <t>狼</t>
         </is>
       </c>
-      <c r="D211" t="inlineStr">
+      <c r="D211" s="0" t="inlineStr">
         <is>
           <t>QQZJ/TPR开局道具。燕子坞家传暗记，可作江湖行走凭证。</t>
         </is>
       </c>
-      <c r="E211" t="n">
-        <v>-1</v>
-      </c>
-      <c r="F211" t="n">
-        <v>-1</v>
-      </c>
-      <c r="G211" t="n">
-        <v>-1</v>
-      </c>
-      <c r="H211" t="n">
-        <v>0</v>
-      </c>
-      <c r="I211" t="n">
-        <v>0</v>
-      </c>
-      <c r="J211" t="n">
-        <v>0</v>
-      </c>
-      <c r="K211" t="n">
-        <v>0</v>
-      </c>
-      <c r="L211" t="n">
-        <v>0</v>
-      </c>
-      <c r="M211" t="n">
-        <v>0</v>
-      </c>
-      <c r="N211" t="n">
-        <v>0</v>
-      </c>
-      <c r="O211" t="n">
-        <v>0</v>
-      </c>
-      <c r="P211" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q211" t="n">
-        <v>0</v>
-      </c>
-      <c r="R211" t="n">
-        <v>0</v>
-      </c>
-      <c r="S211" t="n">
-        <v>0</v>
-      </c>
-      <c r="T211" t="n">
-        <v>0</v>
-      </c>
-      <c r="U211" t="n">
-        <v>0</v>
-      </c>
-      <c r="V211" t="n">
-        <v>0</v>
-      </c>
-      <c r="W211" t="n">
-        <v>0</v>
-      </c>
-      <c r="X211" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y211" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z211" t="n">
-        <v>0</v>
-      </c>
-      <c r="AA211" t="n">
-        <v>0</v>
-      </c>
-      <c r="AB211" t="n">
-        <v>0</v>
-      </c>
-      <c r="AC211" t="n">
-        <v>0</v>
-      </c>
-      <c r="AD211" t="n">
-        <v>0</v>
-      </c>
-      <c r="AE211" t="n">
-        <v>0</v>
-      </c>
-      <c r="AF211" t="n">
-        <v>0</v>
-      </c>
-      <c r="AG211" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH211" t="n">
-        <v>0</v>
-      </c>
-      <c r="AI211" t="n">
-        <v>0</v>
-      </c>
-      <c r="AJ211" t="n">
-        <v>0</v>
-      </c>
-      <c r="AK211" t="n">
-        <v>0</v>
-      </c>
-      <c r="AL211" t="n">
-        <v>0</v>
-      </c>
-      <c r="AM211" t="n">
-        <v>0</v>
-      </c>
-      <c r="AN211" t="n">
-        <v>0</v>
-      </c>
-      <c r="AO211" t="n">
-        <v>0</v>
-      </c>
-      <c r="AP211" t="n">
-        <v>0</v>
-      </c>
-      <c r="AQ211" t="n">
-        <v>0</v>
-      </c>
-      <c r="AR211" t="n">
-        <v>0</v>
-      </c>
-      <c r="AS211" t="n">
-        <v>0</v>
-      </c>
-      <c r="AT211" t="n">
-        <v>0</v>
-      </c>
-      <c r="AU211" t="n">
-        <v>-1</v>
-      </c>
-      <c r="AV211" t="n">
-        <v>0</v>
-      </c>
-      <c r="AW211" t="n">
-        <v>-1</v>
-      </c>
-      <c r="AX211" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
+      <c r="E211" s="0" t="n">
+        <v>-1</v>
+      </c>
+      <c r="F211" s="0" t="n">
+        <v>-1</v>
+      </c>
+      <c r="G211" s="0" t="n">
+        <v>-1</v>
+      </c>
+      <c r="H211" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="I211" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="J211" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="K211" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="L211" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="M211" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="N211" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="O211" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="P211" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q211" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="R211" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="S211" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="T211" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="U211" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="V211" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="W211" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="X211" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y211" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z211" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA211" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB211" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC211" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD211" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE211" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF211" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG211" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH211" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI211" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ211" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK211" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL211" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM211" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN211" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO211" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP211" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ211" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR211" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS211" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT211" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU211" s="0" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AV211" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW211" s="0" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AX211" s="0" t="inlineStr"/>
     </row>
     <row r="212">
-      <c r="A212" t="n">
+      <c r="A212" s="0" t="n">
         <v>207</v>
       </c>
-      <c r="B212" t="inlineStr">
+      <c r="B212" s="0" t="inlineStr">
         <is>
           <t>秦皇照骨镜</t>
         </is>
       </c>
-      <c r="C212" t="inlineStr">
+      <c r="C212" s="0" t="inlineStr">
         <is>
           <t>秦</t>
         </is>
       </c>
-      <c r="D212" t="inlineStr">
+      <c r="D212" s="0" t="inlineStr">
         <is>
           <t>QQZJ/TPR开局道具。古镜一面，据说可照见机关与遗迹线索。</t>
         </is>
       </c>
-      <c r="E212" t="n">
-        <v>-1</v>
-      </c>
-      <c r="F212" t="n">
-        <v>-1</v>
-      </c>
-      <c r="G212" t="n">
-        <v>-1</v>
-      </c>
-      <c r="H212" t="n">
-        <v>0</v>
-      </c>
-      <c r="I212" t="n">
-        <v>0</v>
-      </c>
-      <c r="J212" t="n">
-        <v>0</v>
-      </c>
-      <c r="K212" t="n">
-        <v>0</v>
-      </c>
-      <c r="L212" t="n">
-        <v>0</v>
-      </c>
-      <c r="M212" t="n">
-        <v>0</v>
-      </c>
-      <c r="N212" t="n">
-        <v>0</v>
-      </c>
-      <c r="O212" t="n">
-        <v>0</v>
-      </c>
-      <c r="P212" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q212" t="n">
-        <v>0</v>
-      </c>
-      <c r="R212" t="n">
-        <v>0</v>
-      </c>
-      <c r="S212" t="n">
-        <v>0</v>
-      </c>
-      <c r="T212" t="n">
-        <v>0</v>
-      </c>
-      <c r="U212" t="n">
-        <v>0</v>
-      </c>
-      <c r="V212" t="n">
-        <v>0</v>
-      </c>
-      <c r="W212" t="n">
-        <v>0</v>
-      </c>
-      <c r="X212" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y212" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z212" t="n">
-        <v>0</v>
-      </c>
-      <c r="AA212" t="n">
-        <v>0</v>
-      </c>
-      <c r="AB212" t="n">
-        <v>0</v>
-      </c>
-      <c r="AC212" t="n">
-        <v>0</v>
-      </c>
-      <c r="AD212" t="n">
-        <v>0</v>
-      </c>
-      <c r="AE212" t="n">
-        <v>0</v>
-      </c>
-      <c r="AF212" t="n">
-        <v>0</v>
-      </c>
-      <c r="AG212" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH212" t="n">
-        <v>0</v>
-      </c>
-      <c r="AI212" t="n">
-        <v>0</v>
-      </c>
-      <c r="AJ212" t="n">
-        <v>0</v>
-      </c>
-      <c r="AK212" t="n">
-        <v>0</v>
-      </c>
-      <c r="AL212" t="n">
-        <v>0</v>
-      </c>
-      <c r="AM212" t="n">
-        <v>0</v>
-      </c>
-      <c r="AN212" t="n">
-        <v>0</v>
-      </c>
-      <c r="AO212" t="n">
-        <v>0</v>
-      </c>
-      <c r="AP212" t="n">
-        <v>0</v>
-      </c>
-      <c r="AQ212" t="n">
-        <v>0</v>
-      </c>
-      <c r="AR212" t="n">
-        <v>0</v>
-      </c>
-      <c r="AS212" t="n">
-        <v>0</v>
-      </c>
-      <c r="AT212" t="n">
-        <v>0</v>
-      </c>
-      <c r="AU212" t="n">
-        <v>-1</v>
-      </c>
-      <c r="AV212" t="n">
-        <v>0</v>
-      </c>
-      <c r="AW212" t="n">
-        <v>-1</v>
-      </c>
-      <c r="AX212" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
+      <c r="E212" s="0" t="n">
+        <v>-1</v>
+      </c>
+      <c r="F212" s="0" t="n">
+        <v>-1</v>
+      </c>
+      <c r="G212" s="0" t="n">
+        <v>-1</v>
+      </c>
+      <c r="H212" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="I212" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="J212" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="K212" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="L212" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="M212" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="N212" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="O212" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="P212" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q212" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="R212" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="S212" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="T212" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="U212" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="V212" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="W212" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="X212" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y212" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z212" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA212" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB212" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC212" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD212" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE212" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF212" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG212" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH212" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI212" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ212" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK212" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL212" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM212" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN212" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO212" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP212" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ212" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR212" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS212" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT212" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU212" s="0" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AV212" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW212" s="0" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AX212" s="0" t="inlineStr"/>
     </row>
     <row r="213">
-      <c r="A213" t="n">
+      <c r="A213" s="0" t="n">
         <v>208</v>
       </c>
-      <c r="B213" t="inlineStr">
+      <c r="B213" s="0" t="inlineStr">
         <is>
           <t>洛阳铲</t>
         </is>
       </c>
-      <c r="C213" t="inlineStr">
+      <c r="C213" s="0" t="inlineStr">
         <is>
           <t>铲</t>
         </is>
       </c>
-      <c r="D213" t="inlineStr">
+      <c r="D213" s="0" t="inlineStr">
         <is>
           <t>QQZJ/TPR开局道具。探墓寻物所用器具。</t>
         </is>
       </c>
-      <c r="E213" t="n">
-        <v>-1</v>
-      </c>
-      <c r="F213" t="n">
-        <v>-1</v>
-      </c>
-      <c r="G213" t="n">
-        <v>-1</v>
-      </c>
-      <c r="H213" t="n">
-        <v>0</v>
-      </c>
-      <c r="I213" t="n">
-        <v>0</v>
-      </c>
-      <c r="J213" t="n">
-        <v>0</v>
-      </c>
-      <c r="K213" t="n">
-        <v>0</v>
-      </c>
-      <c r="L213" t="n">
-        <v>0</v>
-      </c>
-      <c r="M213" t="n">
-        <v>0</v>
-      </c>
-      <c r="N213" t="n">
-        <v>0</v>
-      </c>
-      <c r="O213" t="n">
-        <v>0</v>
-      </c>
-      <c r="P213" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q213" t="n">
-        <v>0</v>
-      </c>
-      <c r="R213" t="n">
-        <v>0</v>
-      </c>
-      <c r="S213" t="n">
-        <v>0</v>
-      </c>
-      <c r="T213" t="n">
-        <v>0</v>
-      </c>
-      <c r="U213" t="n">
-        <v>0</v>
-      </c>
-      <c r="V213" t="n">
-        <v>0</v>
-      </c>
-      <c r="W213" t="n">
-        <v>0</v>
-      </c>
-      <c r="X213" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y213" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z213" t="n">
-        <v>0</v>
-      </c>
-      <c r="AA213" t="n">
-        <v>0</v>
-      </c>
-      <c r="AB213" t="n">
-        <v>0</v>
-      </c>
-      <c r="AC213" t="n">
-        <v>0</v>
-      </c>
-      <c r="AD213" t="n">
-        <v>0</v>
-      </c>
-      <c r="AE213" t="n">
-        <v>0</v>
-      </c>
-      <c r="AF213" t="n">
-        <v>0</v>
-      </c>
-      <c r="AG213" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH213" t="n">
-        <v>0</v>
-      </c>
-      <c r="AI213" t="n">
-        <v>0</v>
-      </c>
-      <c r="AJ213" t="n">
-        <v>0</v>
-      </c>
-      <c r="AK213" t="n">
-        <v>0</v>
-      </c>
-      <c r="AL213" t="n">
-        <v>0</v>
-      </c>
-      <c r="AM213" t="n">
-        <v>0</v>
-      </c>
-      <c r="AN213" t="n">
-        <v>0</v>
-      </c>
-      <c r="AO213" t="n">
-        <v>0</v>
-      </c>
-      <c r="AP213" t="n">
-        <v>0</v>
-      </c>
-      <c r="AQ213" t="n">
-        <v>0</v>
-      </c>
-      <c r="AR213" t="n">
-        <v>0</v>
-      </c>
-      <c r="AS213" t="n">
-        <v>0</v>
-      </c>
-      <c r="AT213" t="n">
-        <v>0</v>
-      </c>
-      <c r="AU213" t="n">
-        <v>-1</v>
-      </c>
-      <c r="AV213" t="n">
-        <v>0</v>
-      </c>
-      <c r="AW213" t="n">
-        <v>-1</v>
-      </c>
-      <c r="AX213" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
+      <c r="E213" s="0" t="n">
+        <v>-1</v>
+      </c>
+      <c r="F213" s="0" t="n">
+        <v>-1</v>
+      </c>
+      <c r="G213" s="0" t="n">
+        <v>-1</v>
+      </c>
+      <c r="H213" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="I213" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="J213" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="K213" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="L213" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="M213" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="N213" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="O213" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="P213" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q213" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="R213" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="S213" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="T213" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="U213" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="V213" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="W213" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="X213" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y213" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z213" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA213" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB213" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC213" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD213" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE213" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF213" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG213" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH213" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI213" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ213" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK213" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL213" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM213" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN213" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO213" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP213" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ213" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR213" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS213" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT213" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU213" s="0" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AV213" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW213" s="0" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AX213" s="0" t="inlineStr"/>
     </row>
-    <row r="214">
-      <c r="A214" t="n">
+    <row r="214" s="9">
+      <c r="A214" s="0" t="n">
         <v>209</v>
       </c>
-      <c r="B214" t="inlineStr">
+      <c r="B214" s="0" t="inlineStr">
         <is>
           <t>海月清辉</t>
         </is>
       </c>
-      <c r="C214" t="inlineStr">
+      <c r="C214" s="0" t="inlineStr">
         <is>
           <t>海</t>
         </is>
       </c>
-      <c r="D214" t="inlineStr">
+      <c r="D214" s="0" t="inlineStr">
         <is>
           <t>QQZJ/TPR开局道具。还施水阁所藏清雅珍物。</t>
         </is>
       </c>
-      <c r="E214" t="n">
-        <v>-1</v>
-      </c>
-      <c r="F214" t="n">
-        <v>-1</v>
-      </c>
-      <c r="G214" t="n">
-        <v>-1</v>
-      </c>
-      <c r="H214" t="n">
-        <v>0</v>
-      </c>
-      <c r="I214" t="n">
-        <v>0</v>
-      </c>
-      <c r="J214" t="n">
-        <v>0</v>
-      </c>
-      <c r="K214" t="n">
-        <v>0</v>
-      </c>
-      <c r="L214" t="n">
-        <v>0</v>
-      </c>
-      <c r="M214" t="n">
-        <v>0</v>
-      </c>
-      <c r="N214" t="n">
-        <v>0</v>
-      </c>
-      <c r="O214" t="n">
-        <v>0</v>
-      </c>
-      <c r="P214" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q214" t="n">
-        <v>0</v>
-      </c>
-      <c r="R214" t="n">
-        <v>0</v>
-      </c>
-      <c r="S214" t="n">
-        <v>0</v>
-      </c>
-      <c r="T214" t="n">
-        <v>0</v>
-      </c>
-      <c r="U214" t="n">
-        <v>0</v>
-      </c>
-      <c r="V214" t="n">
-        <v>0</v>
-      </c>
-      <c r="W214" t="n">
-        <v>0</v>
-      </c>
-      <c r="X214" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y214" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z214" t="n">
-        <v>0</v>
-      </c>
-      <c r="AA214" t="n">
-        <v>0</v>
-      </c>
-      <c r="AB214" t="n">
-        <v>0</v>
-      </c>
-      <c r="AC214" t="n">
-        <v>0</v>
-      </c>
-      <c r="AD214" t="n">
-        <v>0</v>
-      </c>
-      <c r="AE214" t="n">
-        <v>0</v>
-      </c>
-      <c r="AF214" t="n">
-        <v>0</v>
-      </c>
-      <c r="AG214" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH214" t="n">
-        <v>0</v>
-      </c>
-      <c r="AI214" t="n">
-        <v>0</v>
-      </c>
-      <c r="AJ214" t="n">
-        <v>0</v>
-      </c>
-      <c r="AK214" t="n">
-        <v>0</v>
-      </c>
-      <c r="AL214" t="n">
-        <v>0</v>
-      </c>
-      <c r="AM214" t="n">
-        <v>0</v>
-      </c>
-      <c r="AN214" t="n">
-        <v>0</v>
-      </c>
-      <c r="AO214" t="n">
-        <v>0</v>
-      </c>
-      <c r="AP214" t="n">
-        <v>0</v>
-      </c>
-      <c r="AQ214" t="n">
-        <v>0</v>
-      </c>
-      <c r="AR214" t="n">
-        <v>0</v>
-      </c>
-      <c r="AS214" t="n">
-        <v>0</v>
-      </c>
-      <c r="AT214" t="n">
-        <v>0</v>
-      </c>
-      <c r="AU214" t="n">
-        <v>-1</v>
-      </c>
-      <c r="AV214" t="n">
-        <v>0</v>
-      </c>
-      <c r="AW214" t="n">
-        <v>-1</v>
-      </c>
-      <c r="AX214" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
+      <c r="E214" s="0" t="n">
+        <v>-1</v>
+      </c>
+      <c r="F214" s="0" t="n">
+        <v>-1</v>
+      </c>
+      <c r="G214" s="0" t="n">
+        <v>-1</v>
+      </c>
+      <c r="H214" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="I214" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="J214" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="K214" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="L214" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="M214" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="N214" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="O214" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="P214" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q214" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="R214" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="S214" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="T214" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="U214" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="V214" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="W214" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="X214" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y214" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z214" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA214" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB214" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC214" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD214" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE214" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF214" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG214" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH214" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI214" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ214" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK214" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL214" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM214" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN214" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO214" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP214" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ214" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR214" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS214" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT214" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU214" s="0" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AV214" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW214" s="0" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AX214" s="0" t="inlineStr"/>
+    </row>
+    <row r="215" s="9">
+      <c r="A215" s="0" t="n">
+        <v>210</v>
+      </c>
+      <c r="B215" s="0" t="inlineStr">
+        <is>
+          <t>金创药</t>
+        </is>
+      </c>
+      <c r="C215" s="0" t="inlineStr">
+        <is>
+          <t>金</t>
+        </is>
+      </c>
+      <c r="D215" s="0" t="inlineStr">
+        <is>
+          <t>QQZJ/TPR开局药品。江湖常见伤药，可恢复少量生命。</t>
+        </is>
+      </c>
+      <c r="E215" s="0" t="n">
+        <v>-1</v>
+      </c>
+      <c r="F215" s="0" t="n">
+        <v>-1</v>
+      </c>
+      <c r="G215" s="0" t="n">
+        <v>-1</v>
+      </c>
+      <c r="H215" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="I215" s="0" t="n">
+        <v>50</v>
+      </c>
+      <c r="J215" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="K215" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="L215" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="M215" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="N215" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="O215" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="P215" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q215" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="R215" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="S215" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="T215" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="U215" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="V215" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="W215" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="X215" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y215" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z215" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA215" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB215" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC215" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD215" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE215" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF215" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG215" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH215" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI215" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ215" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK215" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL215" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM215" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN215" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO215" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP215" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ215" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR215" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS215" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT215" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU215" s="0" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AV215" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW215" s="0" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AX215" s="0" t="inlineStr"/>
+    </row>
+    <row r="216" s="9">
+      <c r="A216" s="0" t="n">
+        <v>211</v>
+      </c>
+      <c r="B216" s="0" t="inlineStr">
+        <is>
+          <t>少阳丹</t>
+        </is>
+      </c>
+      <c r="C216" s="0" t="inlineStr">
+        <is>
+          <t>少</t>
+        </is>
+      </c>
+      <c r="D216" s="0" t="inlineStr">
+        <is>
+          <t>QQZJ/TPR开局药品。温养少阳之气，可恢复少量内力。</t>
+        </is>
+      </c>
+      <c r="E216" s="0" t="n">
+        <v>-1</v>
+      </c>
+      <c r="F216" s="0" t="n">
+        <v>-1</v>
+      </c>
+      <c r="G216" s="0" t="n">
+        <v>-1</v>
+      </c>
+      <c r="H216" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="I216" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="J216" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="K216" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="L216" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="M216" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="N216" s="0" t="n">
+        <v>50</v>
+      </c>
+      <c r="O216" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="P216" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q216" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="R216" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="S216" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="T216" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="U216" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="V216" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="W216" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="X216" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y216" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z216" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA216" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB216" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC216" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD216" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE216" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF216" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG216" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH216" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI216" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ216" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK216" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL216" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM216" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN216" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO216" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP216" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ216" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR216" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS216" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT216" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU216" s="0" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AV216" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW216" s="0" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AX216" s="0" t="inlineStr"/>
+    </row>
+    <row r="217" s="9">
+      <c r="A217" s="0" t="n">
+        <v>212</v>
+      </c>
+      <c r="B217" s="0" t="inlineStr">
+        <is>
+          <t>人参养荣丸</t>
+        </is>
+      </c>
+      <c r="C217" s="0" t="inlineStr">
+        <is>
+          <t>养</t>
+        </is>
+      </c>
+      <c r="D217" s="0" t="inlineStr">
+        <is>
+          <t>QQZJ/TPR开局药品。补气养荣，可恢复生命与内力。</t>
+        </is>
+      </c>
+      <c r="E217" s="0" t="n">
+        <v>-1</v>
+      </c>
+      <c r="F217" s="0" t="n">
+        <v>-1</v>
+      </c>
+      <c r="G217" s="0" t="n">
+        <v>-1</v>
+      </c>
+      <c r="H217" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="I217" s="0" t="n">
+        <v>100</v>
+      </c>
+      <c r="J217" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="K217" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="L217" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="M217" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="N217" s="0" t="n">
+        <v>100</v>
+      </c>
+      <c r="O217" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="P217" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q217" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="R217" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="S217" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="T217" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="U217" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="V217" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="W217" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="X217" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y217" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z217" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA217" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB217" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC217" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD217" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE217" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF217" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG217" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH217" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI217" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ217" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK217" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL217" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM217" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN217" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO217" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP217" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ217" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR217" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS217" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT217" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU217" s="0" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AV217" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW217" s="0" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AX217" s="0" t="inlineStr"/>
+    </row>
+    <row r="218" s="9">
+      <c r="A218" s="0" t="n">
+        <v>213</v>
+      </c>
+      <c r="B218" s="0" t="inlineStr">
+        <is>
+          <t>明玉丹</t>
+        </is>
+      </c>
+      <c r="C218" s="0" t="inlineStr">
+        <is>
+          <t>明</t>
+        </is>
+      </c>
+      <c r="D218" s="0" t="inlineStr">
+        <is>
+          <t>QQZJ/TPR开局服务道具。慕容秋荻处明玉丹服务占位，暂不具备直接药效。</t>
+        </is>
+      </c>
+      <c r="E218" s="0" t="n">
+        <v>-1</v>
+      </c>
+      <c r="F218" s="0" t="n">
+        <v>-1</v>
+      </c>
+      <c r="G218" s="0" t="n">
+        <v>-1</v>
+      </c>
+      <c r="H218" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="I218" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="J218" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="K218" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="L218" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="M218" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="N218" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="O218" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="P218" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q218" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="R218" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="S218" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="T218" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="U218" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="V218" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="W218" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="X218" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y218" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z218" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA218" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB218" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC218" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD218" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE218" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF218" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG218" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH218" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI218" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ218" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK218" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL218" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM218" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN218" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO218" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP218" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ218" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR218" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS218" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT218" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU218" s="0" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AV218" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW218" s="0" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AX218" s="0" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>